<commit_message>
gantt coloreado hasta el 24-sep, con la columna de hoy marcada
- Lo terminado va en el color fuerte de su responsable; lo que va en curso,
  fuerte hasta hoy y claro lo que falta del plan. Antes los estados decian OK
  pero las barras de la 11 a la 15 seguian en color claro.
- La columna del 23 (la ultima sesion antes del examen del jueves 24) lleva
  banda, bordes rojos y la etiqueta HOY; la leyenda explica los colores.
- 23 y 25 terminadas: dataset preparado por paquete (1703 imagenes) y prueba
  temprana del modelo (exactitud en test 0.82), auditadas en feature/modelo-ia.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ficha-tecnica/GANTT_Vixta_actualizado.xlsx
+++ b/docs/ficha-tecnica/GANTT_Vixta_actualizado.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -85,8 +85,26 @@
       <color rgb="FF4B5563"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="7"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFE74C3C"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="23">
+  <fills count="24">
     <fill>
       <patternFill/>
     </fill>
@@ -201,8 +219,13 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD5DAE1"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -302,11 +325,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFE74C3C"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFE74C3C"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD6DBE3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD6DBE3"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -400,6 +437,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -792,6 +844,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="Z3" s="49" t="inlineStr">
+        <is>
+          <t>HOY</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="38" t="inlineStr">
         <is>
@@ -938,7 +997,7 @@
       <c r="Y5" s="1" t="n">
         <v>21</v>
       </c>
-      <c r="Z5" s="1" t="n">
+      <c r="Z5" s="50" t="n">
         <v>23</v>
       </c>
       <c r="AA5" s="1" t="n">
@@ -1076,7 +1135,7 @@
           <t>L</t>
         </is>
       </c>
-      <c r="Z6" s="2" t="inlineStr">
+      <c r="Z6" s="51" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -1190,7 +1249,7 @@
       <c r="W7" s="9" t="n"/>
       <c r="X7" s="9" t="n"/>
       <c r="Y7" s="9" t="n"/>
-      <c r="Z7" s="9" t="n"/>
+      <c r="Z7" s="52" t="n"/>
       <c r="AA7" s="9" t="n"/>
       <c r="AB7" s="9" t="n"/>
       <c r="AC7" s="9" t="n"/>
@@ -1252,7 +1311,7 @@
       <c r="W8" s="14" t="n"/>
       <c r="X8" s="14" t="n"/>
       <c r="Y8" s="14" t="n"/>
-      <c r="Z8" s="14" t="n"/>
+      <c r="Z8" s="52" t="n"/>
       <c r="AA8" s="14" t="n"/>
       <c r="AB8" s="14" t="n"/>
       <c r="AC8" s="14" t="n"/>
@@ -1314,7 +1373,7 @@
       <c r="W9" s="9" t="n"/>
       <c r="X9" s="9" t="n"/>
       <c r="Y9" s="9" t="n"/>
-      <c r="Z9" s="9" t="n"/>
+      <c r="Z9" s="52" t="n"/>
       <c r="AA9" s="9" t="n"/>
       <c r="AB9" s="9" t="n"/>
       <c r="AC9" s="9" t="n"/>
@@ -1376,7 +1435,7 @@
       <c r="W10" s="14" t="n"/>
       <c r="X10" s="14" t="n"/>
       <c r="Y10" s="14" t="n"/>
-      <c r="Z10" s="14" t="n"/>
+      <c r="Z10" s="52" t="n"/>
       <c r="AA10" s="14" t="n"/>
       <c r="AB10" s="14" t="n"/>
       <c r="AC10" s="14" t="n"/>
@@ -1437,12 +1496,12 @@
       <c r="R11" s="9" t="n"/>
       <c r="S11" s="16" t="n"/>
       <c r="T11" s="16" t="n"/>
-      <c r="U11" s="34" t="n"/>
+      <c r="U11" s="16" t="n"/>
       <c r="V11" s="9" t="n"/>
       <c r="W11" s="9" t="n"/>
       <c r="X11" s="9" t="n"/>
       <c r="Y11" s="9" t="n"/>
-      <c r="Z11" s="9" t="n"/>
+      <c r="Z11" s="52" t="n"/>
       <c r="AA11" s="9" t="n"/>
       <c r="AB11" s="9" t="n"/>
       <c r="AC11" s="9" t="n"/>
@@ -1504,7 +1563,7 @@
       <c r="W12" s="14" t="n"/>
       <c r="X12" s="14" t="n"/>
       <c r="Y12" s="14" t="n"/>
-      <c r="Z12" s="14" t="n"/>
+      <c r="Z12" s="52" t="n"/>
       <c r="AA12" s="14" t="n"/>
       <c r="AB12" s="14" t="n"/>
       <c r="AC12" s="14" t="n"/>
@@ -1561,12 +1620,12 @@
       <c r="R13" s="9" t="n"/>
       <c r="S13" s="9" t="n"/>
       <c r="T13" s="15" t="n"/>
-      <c r="U13" s="35" t="n"/>
-      <c r="V13" s="35" t="n"/>
+      <c r="U13" s="15" t="n"/>
+      <c r="V13" s="15" t="n"/>
       <c r="W13" s="9" t="n"/>
       <c r="X13" s="9" t="n"/>
       <c r="Y13" s="9" t="n"/>
-      <c r="Z13" s="9" t="n"/>
+      <c r="Z13" s="52" t="n"/>
       <c r="AA13" s="9" t="n"/>
       <c r="AB13" s="9" t="n"/>
       <c r="AC13" s="9" t="n"/>
@@ -1628,12 +1687,12 @@
       <c r="R14" s="14" t="n"/>
       <c r="S14" s="14" t="n"/>
       <c r="T14" s="14" t="n"/>
-      <c r="U14" s="35" t="n"/>
-      <c r="V14" s="35" t="n"/>
+      <c r="U14" s="15" t="n"/>
+      <c r="V14" s="15" t="n"/>
       <c r="W14" s="14" t="n"/>
       <c r="X14" s="14" t="n"/>
       <c r="Y14" s="14" t="n"/>
-      <c r="Z14" s="14" t="n"/>
+      <c r="Z14" s="52" t="n"/>
       <c r="AA14" s="14" t="n"/>
       <c r="AB14" s="14" t="n"/>
       <c r="AC14" s="14" t="n"/>
@@ -1705,12 +1764,12 @@
       <c r="R15" s="9" t="n"/>
       <c r="S15" s="9" t="n"/>
       <c r="T15" s="16" t="n"/>
-      <c r="U15" s="34" t="n"/>
+      <c r="U15" s="16" t="n"/>
       <c r="V15" s="9" t="n"/>
       <c r="W15" s="9" t="n"/>
       <c r="X15" s="9" t="n"/>
       <c r="Y15" s="9" t="n"/>
-      <c r="Z15" s="9" t="n"/>
+      <c r="Z15" s="52" t="n"/>
       <c r="AA15" s="9" t="n"/>
       <c r="AB15" s="9" t="n"/>
       <c r="AC15" s="9" t="n"/>
@@ -1779,11 +1838,11 @@
       <c r="S16" s="14" t="n"/>
       <c r="T16" s="14" t="n"/>
       <c r="U16" s="14" t="n"/>
-      <c r="V16" s="34" t="n"/>
-      <c r="W16" s="17" t="n"/>
-      <c r="X16" s="17" t="n"/>
-      <c r="Y16" s="17" t="n"/>
-      <c r="Z16" s="17" t="n"/>
+      <c r="V16" s="16" t="n"/>
+      <c r="W16" s="16" t="n"/>
+      <c r="X16" s="16" t="n"/>
+      <c r="Y16" s="16" t="n"/>
+      <c r="Z16" s="53" t="n"/>
       <c r="AA16" s="17" t="n"/>
       <c r="AB16" s="17" t="n"/>
       <c r="AC16" s="17" t="n"/>
@@ -1852,11 +1911,11 @@
       <c r="S17" s="9" t="n"/>
       <c r="T17" s="9" t="n"/>
       <c r="U17" s="9" t="n"/>
-      <c r="V17" s="35" t="n"/>
-      <c r="W17" s="18" t="n"/>
+      <c r="V17" s="15" t="n"/>
+      <c r="W17" s="15" t="n"/>
       <c r="X17" s="9" t="n"/>
       <c r="Y17" s="9" t="n"/>
-      <c r="Z17" s="9" t="n"/>
+      <c r="Z17" s="52" t="n"/>
       <c r="AA17" s="9" t="n"/>
       <c r="AB17" s="9" t="n"/>
       <c r="AC17" s="9" t="n"/>
@@ -1926,10 +1985,10 @@
       <c r="T18" s="14" t="n"/>
       <c r="U18" s="14" t="n"/>
       <c r="V18" s="14" t="n"/>
-      <c r="W18" s="18" t="n"/>
-      <c r="X18" s="18" t="n"/>
+      <c r="W18" s="15" t="n"/>
+      <c r="X18" s="15" t="n"/>
       <c r="Y18" s="14" t="n"/>
-      <c r="Z18" s="14" t="n"/>
+      <c r="Z18" s="52" t="n"/>
       <c r="AA18" s="14" t="n"/>
       <c r="AB18" s="14" t="n"/>
       <c r="AC18" s="14" t="n"/>
@@ -1999,10 +2058,10 @@
       <c r="T19" s="9" t="n"/>
       <c r="U19" s="9" t="n"/>
       <c r="V19" s="44" t="n"/>
-      <c r="W19" s="19" t="n"/>
-      <c r="X19" s="19" t="n"/>
+      <c r="W19" s="44" t="n"/>
+      <c r="X19" s="44" t="n"/>
       <c r="Y19" s="9" t="n"/>
-      <c r="Z19" s="9" t="n"/>
+      <c r="Z19" s="52" t="n"/>
       <c r="AA19" s="9" t="n"/>
       <c r="AB19" s="9" t="n"/>
       <c r="AC19" s="9" t="n"/>
@@ -2075,11 +2134,11 @@
       <c r="S20" s="14" t="n"/>
       <c r="T20" s="14" t="n"/>
       <c r="U20" s="14" t="n"/>
-      <c r="V20" s="34" t="n"/>
-      <c r="W20" s="17" t="n"/>
-      <c r="X20" s="17" t="n"/>
+      <c r="V20" s="16" t="n"/>
+      <c r="W20" s="16" t="n"/>
+      <c r="X20" s="16" t="n"/>
       <c r="Y20" s="14" t="n"/>
-      <c r="Z20" s="14" t="n"/>
+      <c r="Z20" s="52" t="n"/>
       <c r="AA20" s="14" t="n"/>
       <c r="AB20" s="14" t="n"/>
       <c r="AC20" s="14" t="n"/>
@@ -2149,10 +2208,10 @@
       <c r="T21" s="9" t="n"/>
       <c r="U21" s="9" t="n"/>
       <c r="V21" s="9" t="n"/>
-      <c r="W21" s="21" t="n"/>
-      <c r="X21" s="21" t="n"/>
+      <c r="W21" s="31" t="n"/>
+      <c r="X21" s="31" t="n"/>
       <c r="Y21" s="9" t="n"/>
-      <c r="Z21" s="9" t="n"/>
+      <c r="Z21" s="52" t="n"/>
       <c r="AA21" s="9" t="n"/>
       <c r="AB21" s="9" t="n"/>
       <c r="AC21" s="9" t="n"/>
@@ -2210,7 +2269,7 @@
       <c r="W22" s="14" t="n"/>
       <c r="X22" s="14" t="n"/>
       <c r="Y22" s="14" t="n"/>
-      <c r="Z22" s="25" t="n"/>
+      <c r="Z22" s="54" t="n"/>
       <c r="AA22" s="14" t="n"/>
       <c r="AB22" s="14" t="n"/>
       <c r="AC22" s="14" t="n"/>
@@ -2281,8 +2340,8 @@
       <c r="V23" s="9" t="n"/>
       <c r="W23" s="9" t="n"/>
       <c r="X23" s="9" t="n"/>
-      <c r="Y23" s="21" t="n"/>
-      <c r="Z23" s="21" t="n"/>
+      <c r="Y23" s="31" t="n"/>
+      <c r="Z23" s="55" t="n"/>
       <c r="AA23" s="21" t="n"/>
       <c r="AB23" s="21" t="n"/>
       <c r="AC23" s="21" t="n"/>
@@ -2295,6 +2354,16 @@
       <c r="AJ23" s="9" t="n"/>
       <c r="AK23" s="9" t="n"/>
       <c r="AL23" s="9" t="n"/>
+      <c r="AO23" s="29" t="inlineStr">
+        <is>
+          <t>Colores</t>
+        </is>
+      </c>
+      <c r="AP23" s="30" t="inlineStr">
+        <is>
+          <t>Color fuerte: lo hecho hasta hoy · color claro: lo que falta del plan</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="25.95" customHeight="1" s="37">
       <c r="A24" s="10" t="n">
@@ -2344,7 +2413,7 @@
       <c r="W24" s="14" t="n"/>
       <c r="X24" s="14" t="n"/>
       <c r="Y24" s="14" t="n"/>
-      <c r="Z24" s="14" t="n"/>
+      <c r="Z24" s="52" t="n"/>
       <c r="AA24" s="14" t="n"/>
       <c r="AB24" s="14" t="n"/>
       <c r="AC24" s="14" t="n"/>
@@ -2357,6 +2426,16 @@
       <c r="AJ24" s="17" t="n"/>
       <c r="AK24" s="14" t="n"/>
       <c r="AL24" s="14" t="n"/>
+      <c r="AO24" s="29" t="inlineStr">
+        <is>
+          <t>Hoy</t>
+        </is>
+      </c>
+      <c r="AP24" s="30" t="inlineStr">
+        <is>
+          <t>jueves 24-sep-2026 · columna del 23-sep, la última sesión que no pasa de hoy</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="25.95" customHeight="1" s="37">
       <c r="A25" s="3" t="n">
@@ -2409,8 +2488,8 @@
       <c r="V25" s="9" t="n"/>
       <c r="W25" s="9" t="n"/>
       <c r="X25" s="9" t="n"/>
-      <c r="Y25" s="26" t="n"/>
-      <c r="Z25" s="26" t="n"/>
+      <c r="Y25" s="32" t="n"/>
+      <c r="Z25" s="56" t="n"/>
       <c r="AA25" s="26" t="n"/>
       <c r="AB25" s="26" t="n"/>
       <c r="AC25" s="9" t="n"/>
@@ -2472,7 +2551,7 @@
       <c r="W26" s="14" t="n"/>
       <c r="X26" s="14" t="n"/>
       <c r="Y26" s="14" t="n"/>
-      <c r="Z26" s="14" t="n"/>
+      <c r="Z26" s="52" t="n"/>
       <c r="AA26" s="14" t="n"/>
       <c r="AB26" s="14" t="n"/>
       <c r="AC26" s="26" t="n"/>
@@ -2534,7 +2613,7 @@
       <c r="W27" s="9" t="n"/>
       <c r="X27" s="9" t="n"/>
       <c r="Y27" s="9" t="n"/>
-      <c r="Z27" s="9" t="n"/>
+      <c r="Z27" s="52" t="n"/>
       <c r="AA27" s="9" t="n"/>
       <c r="AB27" s="9" t="n"/>
       <c r="AC27" s="9" t="n"/>
@@ -2595,12 +2674,12 @@
       <c r="R28" s="14" t="n"/>
       <c r="S28" s="14" t="n"/>
       <c r="T28" s="15" t="n"/>
-      <c r="U28" s="35" t="n"/>
+      <c r="U28" s="15" t="n"/>
       <c r="V28" s="14" t="n"/>
       <c r="W28" s="14" t="n"/>
       <c r="X28" s="14" t="n"/>
       <c r="Y28" s="14" t="n"/>
-      <c r="Z28" s="14" t="n"/>
+      <c r="Z28" s="52" t="n"/>
       <c r="AA28" s="14" t="n"/>
       <c r="AB28" s="14" t="n"/>
       <c r="AC28" s="14" t="n"/>
@@ -2641,7 +2720,7 @@
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="H29" s="9" t="n"/>
@@ -2658,11 +2737,11 @@
       <c r="S29" s="9" t="n"/>
       <c r="T29" s="9" t="n"/>
       <c r="U29" s="9" t="n"/>
-      <c r="V29" s="35" t="n"/>
-      <c r="W29" s="18" t="n"/>
+      <c r="V29" s="15" t="n"/>
+      <c r="W29" s="15" t="n"/>
       <c r="X29" s="9" t="n"/>
       <c r="Y29" s="9" t="n"/>
-      <c r="Z29" s="9" t="n"/>
+      <c r="Z29" s="52" t="n"/>
       <c r="AA29" s="9" t="n"/>
       <c r="AB29" s="9" t="n"/>
       <c r="AC29" s="9" t="n"/>
@@ -2722,9 +2801,9 @@
       <c r="U30" s="14" t="n"/>
       <c r="V30" s="14" t="n"/>
       <c r="W30" s="14" t="n"/>
-      <c r="X30" s="27" t="n"/>
-      <c r="Y30" s="27" t="n"/>
-      <c r="Z30" s="27" t="n"/>
+      <c r="X30" s="8" t="n"/>
+      <c r="Y30" s="8" t="n"/>
+      <c r="Z30" s="57" t="n"/>
       <c r="AA30" s="27" t="n"/>
       <c r="AB30" s="27" t="n"/>
       <c r="AC30" s="14" t="n"/>
@@ -2765,7 +2844,7 @@
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>En espera</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="H31" s="9" t="n"/>
@@ -2784,9 +2863,9 @@
       <c r="U31" s="9" t="n"/>
       <c r="V31" s="9" t="n"/>
       <c r="W31" s="9" t="n"/>
-      <c r="X31" s="18" t="n"/>
-      <c r="Y31" s="18" t="n"/>
-      <c r="Z31" s="9" t="n"/>
+      <c r="X31" s="15" t="n"/>
+      <c r="Y31" s="15" t="n"/>
+      <c r="Z31" s="52" t="n"/>
       <c r="AA31" s="9" t="n"/>
       <c r="AB31" s="9" t="n"/>
       <c r="AC31" s="9" t="n"/>
@@ -2848,7 +2927,7 @@
       <c r="W32" s="14" t="n"/>
       <c r="X32" s="14" t="n"/>
       <c r="Y32" s="14" t="n"/>
-      <c r="Z32" s="14" t="n"/>
+      <c r="Z32" s="52" t="n"/>
       <c r="AA32" s="14" t="n"/>
       <c r="AB32" s="14" t="n"/>
       <c r="AC32" s="18" t="n"/>
@@ -2910,7 +2989,7 @@
       <c r="W33" s="9" t="n"/>
       <c r="X33" s="9" t="n"/>
       <c r="Y33" s="9" t="n"/>
-      <c r="Z33" s="9" t="n"/>
+      <c r="Z33" s="52" t="n"/>
       <c r="AA33" s="9" t="n"/>
       <c r="AB33" s="9" t="n"/>
       <c r="AC33" s="9" t="n"/>
@@ -2972,7 +3051,7 @@
       <c r="W34" s="14" t="n"/>
       <c r="X34" s="14" t="n"/>
       <c r="Y34" s="14" t="n"/>
-      <c r="Z34" s="14" t="n"/>
+      <c r="Z34" s="52" t="n"/>
       <c r="AA34" s="14" t="n"/>
       <c r="AB34" s="14" t="n"/>
       <c r="AC34" s="14" t="n"/>
@@ -3034,7 +3113,7 @@
       <c r="W35" s="9" t="n"/>
       <c r="X35" s="9" t="n"/>
       <c r="Y35" s="9" t="n"/>
-      <c r="Z35" s="9" t="n"/>
+      <c r="Z35" s="52" t="n"/>
       <c r="AA35" s="9" t="n"/>
       <c r="AB35" s="9" t="n"/>
       <c r="AC35" s="9" t="n"/>
@@ -3100,7 +3179,7 @@
       <c r="W36" s="14" t="n"/>
       <c r="X36" s="14" t="n"/>
       <c r="Y36" s="14" t="n"/>
-      <c r="Z36" s="14" t="n"/>
+      <c r="Z36" s="52" t="n"/>
       <c r="AA36" s="14" t="n"/>
       <c r="AB36" s="14" t="n"/>
       <c r="AC36" s="14" t="n"/>
@@ -3162,7 +3241,7 @@
       <c r="W37" s="9" t="n"/>
       <c r="X37" s="9" t="n"/>
       <c r="Y37" s="9" t="n"/>
-      <c r="Z37" s="9" t="n"/>
+      <c r="Z37" s="52" t="n"/>
       <c r="AA37" s="9" t="n"/>
       <c r="AB37" s="9" t="n"/>
       <c r="AC37" s="9" t="n"/>
@@ -3224,7 +3303,7 @@
       <c r="W38" s="14" t="n"/>
       <c r="X38" s="14" t="n"/>
       <c r="Y38" s="14" t="n"/>
-      <c r="Z38" s="14" t="n"/>
+      <c r="Z38" s="52" t="n"/>
       <c r="AA38" s="14" t="n"/>
       <c r="AB38" s="14" t="n"/>
       <c r="AC38" s="14" t="n"/>
@@ -3286,7 +3365,7 @@
       <c r="W39" s="9" t="n"/>
       <c r="X39" s="9" t="n"/>
       <c r="Y39" s="9" t="n"/>
-      <c r="Z39" s="9" t="n"/>
+      <c r="Z39" s="52" t="n"/>
       <c r="AA39" s="9" t="n"/>
       <c r="AB39" s="9" t="n"/>
       <c r="AC39" s="9" t="n"/>
@@ -3348,7 +3427,7 @@
       <c r="W40" s="14" t="n"/>
       <c r="X40" s="14" t="n"/>
       <c r="Y40" s="14" t="n"/>
-      <c r="Z40" s="14" t="n"/>
+      <c r="Z40" s="52" t="n"/>
       <c r="AA40" s="14" t="n"/>
       <c r="AB40" s="14" t="n"/>
       <c r="AC40" s="14" t="n"/>
@@ -3410,7 +3489,7 @@
       <c r="W41" s="9" t="n"/>
       <c r="X41" s="9" t="n"/>
       <c r="Y41" s="9" t="n"/>
-      <c r="Z41" s="9" t="n"/>
+      <c r="Z41" s="52" t="n"/>
       <c r="AA41" s="9" t="n"/>
       <c r="AB41" s="9" t="n"/>
       <c r="AC41" s="9" t="n"/>

</xml_diff>